<commit_message>
Se agregó link de documentación oficial de GIT
</commit_message>
<xml_diff>
--- a/links de interes.xlsx
+++ b/links de interes.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="67">
   <si>
     <t>Enlace</t>
   </si>
@@ -202,6 +202,24 @@
   </si>
   <si>
     <t>Servidor para subir aplicaciones</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=QCw0L6FupQ0</t>
+  </si>
+  <si>
+    <t>Curso de Bootstrap desde Cero</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> HTML y CSS - Curso Desde Cero</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=XqFR2lqBYPs</t>
+  </si>
+  <si>
+    <t>https://git-scm.com/book/es/v2/Fundamentos-de-Git-Obteniendo-un-repositorio-Git</t>
+  </si>
+  <si>
+    <t>Documentación oficial git</t>
   </si>
 </sst>
 </file>
@@ -531,7 +549,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:C33"/>
+  <dimension ref="B2:C36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="64.28515625" bestFit="1" customWidth="1"/>
@@ -556,279 +574,306 @@
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
-        <v>4</v>
+        <v>64</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="C11" t="s">
-        <v>19</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="C13" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
+      </c>
+      <c r="C14" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C28" t="s">
-        <v>51</v>
+        <v>46</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C29" t="s">
-        <v>53</v>
+        <v>47</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B30" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C30" t="s">
-        <v>55</v>
+        <v>48</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C31" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="32" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B32" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C32" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C33" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B34" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B35" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C35" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B36" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C36" t="s">
         <v>60</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1"/>
-    <hyperlink ref="B4" r:id="rId2"/>
-    <hyperlink ref="B5" r:id="rId3"/>
-    <hyperlink ref="B6" r:id="rId4"/>
-    <hyperlink ref="B7" r:id="rId5"/>
-    <hyperlink ref="B8" r:id="rId6"/>
-    <hyperlink ref="B9" r:id="rId7"/>
-    <hyperlink ref="B10" r:id="rId8"/>
-    <hyperlink ref="B11" r:id="rId9"/>
-    <hyperlink ref="B12" r:id="rId10"/>
-    <hyperlink ref="B13" r:id="rId11"/>
-    <hyperlink ref="B14" r:id="rId12"/>
-    <hyperlink ref="B15" r:id="rId13"/>
-    <hyperlink ref="B16" r:id="rId14"/>
-    <hyperlink ref="B17" r:id="rId15"/>
-    <hyperlink ref="B18" r:id="rId16"/>
-    <hyperlink ref="B19" r:id="rId17"/>
-    <hyperlink ref="B20" r:id="rId18"/>
-    <hyperlink ref="B21" r:id="rId19"/>
-    <hyperlink ref="B22" r:id="rId20"/>
-    <hyperlink ref="B23" r:id="rId21"/>
-    <hyperlink ref="B24" r:id="rId22"/>
-    <hyperlink ref="B25" r:id="rId23"/>
-    <hyperlink ref="B26" r:id="rId24"/>
-    <hyperlink ref="B27" r:id="rId25"/>
-    <hyperlink ref="B28" r:id="rId26"/>
-    <hyperlink ref="B29" r:id="rId27"/>
-    <hyperlink ref="B30" r:id="rId28"/>
-    <hyperlink ref="B31" r:id="rId29"/>
-    <hyperlink ref="B32" r:id="rId30"/>
-    <hyperlink ref="B33" r:id="rId31"/>
+    <hyperlink ref="B5" r:id="rId2"/>
+    <hyperlink ref="B6" r:id="rId3"/>
+    <hyperlink ref="B7" r:id="rId4"/>
+    <hyperlink ref="B8" r:id="rId5"/>
+    <hyperlink ref="B9" r:id="rId6"/>
+    <hyperlink ref="B10" r:id="rId7"/>
+    <hyperlink ref="B12" r:id="rId8"/>
+    <hyperlink ref="B13" r:id="rId9"/>
+    <hyperlink ref="B14" r:id="rId10"/>
+    <hyperlink ref="B15" r:id="rId11"/>
+    <hyperlink ref="B16" r:id="rId12"/>
+    <hyperlink ref="B17" r:id="rId13"/>
+    <hyperlink ref="B18" r:id="rId14"/>
+    <hyperlink ref="B20" r:id="rId15"/>
+    <hyperlink ref="B21" r:id="rId16"/>
+    <hyperlink ref="B22" r:id="rId17"/>
+    <hyperlink ref="B23" r:id="rId18"/>
+    <hyperlink ref="B24" r:id="rId19"/>
+    <hyperlink ref="B25" r:id="rId20"/>
+    <hyperlink ref="B26" r:id="rId21"/>
+    <hyperlink ref="B27" r:id="rId22"/>
+    <hyperlink ref="B28" r:id="rId23"/>
+    <hyperlink ref="B29" r:id="rId24"/>
+    <hyperlink ref="B30" r:id="rId25"/>
+    <hyperlink ref="B31" r:id="rId26"/>
+    <hyperlink ref="B32" r:id="rId27"/>
+    <hyperlink ref="B33" r:id="rId28"/>
+    <hyperlink ref="B34" r:id="rId29"/>
+    <hyperlink ref="B35" r:id="rId30"/>
+    <hyperlink ref="B36" r:id="rId31"/>
+    <hyperlink ref="B19" r:id="rId32"/>
+    <hyperlink ref="B4" r:id="rId33"/>
+    <hyperlink ref="B11" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId32"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId35"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ejemplo de responsividad con css - grupo 2
</commit_message>
<xml_diff>
--- a/links de interes.xlsx
+++ b/links de interes.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="70">
   <si>
     <t>Enlace</t>
   </si>
@@ -220,6 +220,15 @@
   </si>
   <si>
     <t>Documentación oficial git</t>
+  </si>
+  <si>
+    <t>https://www.w3schools.com/css/css_rwd_intro.asp</t>
+  </si>
+  <si>
+    <t>Ejemplo de responsividad con css</t>
+  </si>
+  <si>
+    <t>Escritura de código más rapida en visual studio code - snipets</t>
   </si>
 </sst>
 </file>
@@ -549,7 +558,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:C36"/>
+  <dimension ref="B2:C38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="64.28515625" bestFit="1" customWidth="1"/>
@@ -582,199 +591,199 @@
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
-        <v>65</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>66</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="C12" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
+      </c>
+      <c r="C15" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
-        <v>26</v>
+        <v>67</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>27</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>62</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>45</v>
@@ -782,98 +791,116 @@
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B30" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C31" t="s">
-        <v>51</v>
+        <v>47</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B32" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C32" t="s">
-        <v>53</v>
+        <v>48</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C33" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C34" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C35" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C36" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B37" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C37" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B38" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C38" t="s">
         <v>60</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1"/>
-    <hyperlink ref="B5" r:id="rId2"/>
-    <hyperlink ref="B6" r:id="rId3"/>
-    <hyperlink ref="B7" r:id="rId4"/>
-    <hyperlink ref="B8" r:id="rId5"/>
-    <hyperlink ref="B9" r:id="rId6"/>
-    <hyperlink ref="B10" r:id="rId7"/>
-    <hyperlink ref="B12" r:id="rId8"/>
-    <hyperlink ref="B13" r:id="rId9"/>
-    <hyperlink ref="B14" r:id="rId10"/>
-    <hyperlink ref="B15" r:id="rId11"/>
-    <hyperlink ref="B16" r:id="rId12"/>
-    <hyperlink ref="B17" r:id="rId13"/>
-    <hyperlink ref="B18" r:id="rId14"/>
-    <hyperlink ref="B20" r:id="rId15"/>
-    <hyperlink ref="B21" r:id="rId16"/>
-    <hyperlink ref="B22" r:id="rId17"/>
-    <hyperlink ref="B23" r:id="rId18"/>
-    <hyperlink ref="B24" r:id="rId19"/>
-    <hyperlink ref="B25" r:id="rId20"/>
-    <hyperlink ref="B26" r:id="rId21"/>
-    <hyperlink ref="B27" r:id="rId22"/>
-    <hyperlink ref="B28" r:id="rId23"/>
-    <hyperlink ref="B29" r:id="rId24"/>
-    <hyperlink ref="B30" r:id="rId25"/>
-    <hyperlink ref="B31" r:id="rId26"/>
-    <hyperlink ref="B32" r:id="rId27"/>
-    <hyperlink ref="B33" r:id="rId28"/>
-    <hyperlink ref="B34" r:id="rId29"/>
-    <hyperlink ref="B35" r:id="rId30"/>
-    <hyperlink ref="B36" r:id="rId31"/>
-    <hyperlink ref="B19" r:id="rId32"/>
+    <hyperlink ref="B6" r:id="rId2"/>
+    <hyperlink ref="B7" r:id="rId3"/>
+    <hyperlink ref="B8" r:id="rId4"/>
+    <hyperlink ref="B9" r:id="rId5"/>
+    <hyperlink ref="B10" r:id="rId6"/>
+    <hyperlink ref="B11" r:id="rId7"/>
+    <hyperlink ref="B13" r:id="rId8"/>
+    <hyperlink ref="B14" r:id="rId9"/>
+    <hyperlink ref="B15" r:id="rId10"/>
+    <hyperlink ref="B16" r:id="rId11"/>
+    <hyperlink ref="B18" r:id="rId12"/>
+    <hyperlink ref="B19" r:id="rId13"/>
+    <hyperlink ref="B20" r:id="rId14"/>
+    <hyperlink ref="B22" r:id="rId15"/>
+    <hyperlink ref="B23" r:id="rId16"/>
+    <hyperlink ref="B24" r:id="rId17"/>
+    <hyperlink ref="B25" r:id="rId18"/>
+    <hyperlink ref="B26" r:id="rId19"/>
+    <hyperlink ref="B27" r:id="rId20"/>
+    <hyperlink ref="B28" r:id="rId21"/>
+    <hyperlink ref="B29" r:id="rId22"/>
+    <hyperlink ref="B30" r:id="rId23"/>
+    <hyperlink ref="B31" r:id="rId24"/>
+    <hyperlink ref="B32" r:id="rId25"/>
+    <hyperlink ref="B33" r:id="rId26"/>
+    <hyperlink ref="B34" r:id="rId27"/>
+    <hyperlink ref="B35" r:id="rId28"/>
+    <hyperlink ref="B36" r:id="rId29"/>
+    <hyperlink ref="B37" r:id="rId30"/>
+    <hyperlink ref="B38" r:id="rId31"/>
+    <hyperlink ref="B21" r:id="rId32"/>
     <hyperlink ref="B4" r:id="rId33"/>
-    <hyperlink ref="B11" r:id="rId34"/>
+    <hyperlink ref="B12" r:id="rId34"/>
+    <hyperlink ref="B17" r:id="rId35"/>
+    <hyperlink ref="B5" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId35"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId37"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualización de archivo con links de interes
</commit_message>
<xml_diff>
--- a/links de interes.xlsx
+++ b/links de interes.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="80">
   <si>
     <t>Enlace</t>
   </si>
@@ -247,6 +247,18 @@
   </si>
   <si>
     <t>Libro js, bunisimo</t>
+  </si>
+  <si>
+    <t>https://learngitbranching.js.org/?utm_source=chatgpt.com&amp;locale=es_AR</t>
+  </si>
+  <si>
+    <t>Herramienta para aprender GIT de forma visual</t>
+  </si>
+  <si>
+    <t>https://ohmygit.org/?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>Aprender git jugado</t>
   </si>
 </sst>
 </file>
@@ -291,10 +303,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -576,7 +591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:C41"/>
+  <dimension ref="B2:C43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="64.28515625" bestFit="1" customWidth="1"/>
@@ -671,153 +686,153 @@
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B13" s="1" t="s">
-        <v>16</v>
+    <row r="13" spans="2:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="3" t="s">
+        <v>76</v>
       </c>
       <c r="C13" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B14" s="1" t="s">
-        <v>18</v>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>78</v>
       </c>
       <c r="C14" t="s">
-        <v>19</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="C16" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>68</v>
+        <v>20</v>
+      </c>
+      <c r="C17" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
-        <v>26</v>
+        <v>67</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>27</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>62</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B30" s="1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>45</v>
@@ -825,81 +840,97 @@
     </row>
     <row r="32" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B32" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34" s="1" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>75</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C36" t="s">
-        <v>51</v>
+        <v>74</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C37" t="s">
-        <v>53</v>
+        <v>70</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C38" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C39" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="40" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C40" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C41" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B42" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C42" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B43" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C43" t="s">
         <v>60</v>
       </c>
     </row>
@@ -912,40 +943,42 @@
     <hyperlink ref="B9" r:id="rId5"/>
     <hyperlink ref="B10" r:id="rId6"/>
     <hyperlink ref="B11" r:id="rId7"/>
-    <hyperlink ref="B13" r:id="rId8"/>
-    <hyperlink ref="B14" r:id="rId9"/>
-    <hyperlink ref="B15" r:id="rId10"/>
-    <hyperlink ref="B16" r:id="rId11"/>
-    <hyperlink ref="B18" r:id="rId12"/>
-    <hyperlink ref="B19" r:id="rId13"/>
-    <hyperlink ref="B20" r:id="rId14"/>
-    <hyperlink ref="B22" r:id="rId15"/>
-    <hyperlink ref="B23" r:id="rId16"/>
-    <hyperlink ref="B24" r:id="rId17"/>
-    <hyperlink ref="B25" r:id="rId18"/>
-    <hyperlink ref="B26" r:id="rId19"/>
-    <hyperlink ref="B27" r:id="rId20"/>
-    <hyperlink ref="B28" r:id="rId21"/>
-    <hyperlink ref="B29" r:id="rId22"/>
-    <hyperlink ref="B30" r:id="rId23"/>
-    <hyperlink ref="B31" r:id="rId24"/>
-    <hyperlink ref="B32" r:id="rId25"/>
-    <hyperlink ref="B36" r:id="rId26"/>
-    <hyperlink ref="B37" r:id="rId27"/>
-    <hyperlink ref="B38" r:id="rId28"/>
-    <hyperlink ref="B39" r:id="rId29"/>
-    <hyperlink ref="B40" r:id="rId30"/>
-    <hyperlink ref="B41" r:id="rId31"/>
-    <hyperlink ref="B21" r:id="rId32"/>
+    <hyperlink ref="B15" r:id="rId8"/>
+    <hyperlink ref="B16" r:id="rId9"/>
+    <hyperlink ref="B17" r:id="rId10"/>
+    <hyperlink ref="B18" r:id="rId11"/>
+    <hyperlink ref="B20" r:id="rId12"/>
+    <hyperlink ref="B21" r:id="rId13"/>
+    <hyperlink ref="B22" r:id="rId14"/>
+    <hyperlink ref="B24" r:id="rId15"/>
+    <hyperlink ref="B25" r:id="rId16"/>
+    <hyperlink ref="B26" r:id="rId17"/>
+    <hyperlink ref="B27" r:id="rId18"/>
+    <hyperlink ref="B28" r:id="rId19"/>
+    <hyperlink ref="B29" r:id="rId20"/>
+    <hyperlink ref="B30" r:id="rId21"/>
+    <hyperlink ref="B31" r:id="rId22"/>
+    <hyperlink ref="B32" r:id="rId23"/>
+    <hyperlink ref="B33" r:id="rId24"/>
+    <hyperlink ref="B34" r:id="rId25"/>
+    <hyperlink ref="B38" r:id="rId26"/>
+    <hyperlink ref="B39" r:id="rId27"/>
+    <hyperlink ref="B40" r:id="rId28"/>
+    <hyperlink ref="B41" r:id="rId29"/>
+    <hyperlink ref="B42" r:id="rId30"/>
+    <hyperlink ref="B43" r:id="rId31"/>
+    <hyperlink ref="B23" r:id="rId32"/>
     <hyperlink ref="B4" r:id="rId33"/>
     <hyperlink ref="B12" r:id="rId34"/>
-    <hyperlink ref="B17" r:id="rId35"/>
+    <hyperlink ref="B19" r:id="rId35"/>
     <hyperlink ref="B5" r:id="rId36"/>
-    <hyperlink ref="B35" r:id="rId37"/>
-    <hyperlink ref="B33" r:id="rId38"/>
-    <hyperlink ref="B34" r:id="rId39"/>
+    <hyperlink ref="B37" r:id="rId37"/>
+    <hyperlink ref="B35" r:id="rId38"/>
+    <hyperlink ref="B36" r:id="rId39"/>
+    <hyperlink ref="B13" r:id="rId40"/>
+    <hyperlink ref="B14" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId40"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId42"/>
 </worksheet>
 </file>
</xml_diff>